<commit_message>
Update OpenF1 lightweight source closure artifacts
</commit_message>
<xml_diff>
--- a/latest/openf1_lightweight_source_closure/F1_OpenF1_Lightweight_Source_Closure_Summary.xlsx
+++ b/latest/openf1_lightweight_source_closure/F1_OpenF1_Lightweight_Source_Closure_Summary.xlsx
@@ -458,7 +458,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6501</v>
+        <v>7090</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,7 +486,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3870</v>
+        <v>4135</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>205981</v>
+        <v>305384</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>30278</v>
+        <v>26790</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3914</v>
+        <v>4179</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>322</v>
+        <v>553</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>242</v>
+        <v>220</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1142</v>
+        <v>1057</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -682,7 +682,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>413</v>
+        <v>465</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1941,11 +1941,11 @@
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -2145,11 +2145,11 @@
         <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>0</v>
+        <v>265</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -2247,11 +2247,11 @@
         <v>1</v>
       </c>
       <c r="G45" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -2315,11 +2315,11 @@
         <v>1</v>
       </c>
       <c r="G47" t="n">
-        <v>0</v>
+        <v>559</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -2349,11 +2349,11 @@
         <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -2417,11 +2417,11 @@
         <v>1</v>
       </c>
       <c r="G50" t="n">
-        <v>0</v>
+        <v>341</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -2451,11 +2451,11 @@
         <v>1</v>
       </c>
       <c r="G51" t="n">
-        <v>0</v>
+        <v>290</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -2553,11 +2553,11 @@
         <v>1</v>
       </c>
       <c r="G54" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -3063,11 +3063,11 @@
         <v>1</v>
       </c>
       <c r="G69" t="n">
-        <v>86</v>
+        <v>0</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -3165,11 +3165,11 @@
         <v>1</v>
       </c>
       <c r="G72" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -3199,11 +3199,11 @@
         <v>1</v>
       </c>
       <c r="G73" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -3233,11 +3233,11 @@
         <v>1</v>
       </c>
       <c r="G74" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -3267,11 +3267,11 @@
         <v>1</v>
       </c>
       <c r="G75" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -3335,11 +3335,11 @@
         <v>1</v>
       </c>
       <c r="G77" t="n">
-        <v>473</v>
+        <v>0</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -3369,11 +3369,11 @@
         <v>1</v>
       </c>
       <c r="G78" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -3471,11 +3471,11 @@
         <v>1</v>
       </c>
       <c r="G81" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -3505,11 +3505,11 @@
         <v>1</v>
       </c>
       <c r="G82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -3539,11 +3539,11 @@
         <v>1</v>
       </c>
       <c r="G83" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -3573,11 +3573,11 @@
         <v>1</v>
       </c>
       <c r="G84" t="n">
-        <v>109</v>
+        <v>0</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -3777,11 +3777,11 @@
         <v>1</v>
       </c>
       <c r="G90" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -3845,11 +3845,11 @@
         <v>1</v>
       </c>
       <c r="G92" t="n">
-        <v>0</v>
+        <v>148</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -3879,11 +3879,11 @@
         <v>1</v>
       </c>
       <c r="G93" t="n">
-        <v>0</v>
+        <v>169</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -3913,11 +3913,11 @@
         <v>1</v>
       </c>
       <c r="G94" t="n">
-        <v>0</v>
+        <v>22276</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -3947,11 +3947,11 @@
         <v>1</v>
       </c>
       <c r="G95" t="n">
-        <v>0</v>
+        <v>531</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -3981,11 +3981,11 @@
         <v>1</v>
       </c>
       <c r="G96" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -4015,11 +4015,11 @@
         <v>1</v>
       </c>
       <c r="G97" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -4083,11 +4083,11 @@
         <v>1</v>
       </c>
       <c r="G99" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -4151,11 +4151,11 @@
         <v>1</v>
       </c>
       <c r="G101" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -4185,11 +4185,11 @@
         <v>1</v>
       </c>
       <c r="G102" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -4253,11 +4253,11 @@
         <v>1</v>
       </c>
       <c r="G104" t="n">
-        <v>779</v>
+        <v>0</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4287,11 +4287,11 @@
         <v>1</v>
       </c>
       <c r="G105" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4389,11 +4389,11 @@
         <v>1</v>
       </c>
       <c r="G108" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4457,11 +4457,11 @@
         <v>1</v>
       </c>
       <c r="G110" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4491,11 +4491,11 @@
         <v>1</v>
       </c>
       <c r="G111" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4559,11 +4559,11 @@
         <v>1</v>
       </c>
       <c r="G113" t="n">
-        <v>1041</v>
+        <v>0</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4593,11 +4593,11 @@
         <v>1</v>
       </c>
       <c r="G114" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4627,11 +4627,11 @@
         <v>1</v>
       </c>
       <c r="G115" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4661,11 +4661,11 @@
         <v>1</v>
       </c>
       <c r="G116" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4695,11 +4695,11 @@
         <v>1</v>
       </c>
       <c r="G117" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4763,11 +4763,11 @@
         <v>1</v>
       </c>
       <c r="G119" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4797,11 +4797,11 @@
         <v>1</v>
       </c>
       <c r="G120" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4831,11 +4831,11 @@
         <v>1</v>
       </c>
       <c r="G121" t="n">
-        <v>9019</v>
+        <v>0</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4865,11 +4865,11 @@
         <v>1</v>
       </c>
       <c r="G122" t="n">
-        <v>351</v>
+        <v>0</v>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4899,11 +4899,11 @@
         <v>1</v>
       </c>
       <c r="G123" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4933,11 +4933,11 @@
         <v>1</v>
       </c>
       <c r="G124" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -5307,11 +5307,11 @@
         <v>1</v>
       </c>
       <c r="G135" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -5375,11 +5375,11 @@
         <v>1</v>
       </c>
       <c r="G137" t="n">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -5409,11 +5409,11 @@
         <v>1</v>
       </c>
       <c r="G138" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -5443,11 +5443,11 @@
         <v>1</v>
       </c>
       <c r="G139" t="n">
-        <v>0</v>
+        <v>20663</v>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -5477,11 +5477,11 @@
         <v>1</v>
       </c>
       <c r="G140" t="n">
-        <v>0</v>
+        <v>524</v>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -5511,11 +5511,11 @@
         <v>1</v>
       </c>
       <c r="G141" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -5545,11 +5545,11 @@
         <v>1</v>
       </c>
       <c r="G142" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -5613,7 +5613,7 @@
         <v>1</v>
       </c>
       <c r="G144" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="H144" t="inlineStr">
         <is>
@@ -6089,11 +6089,11 @@
         <v>1</v>
       </c>
       <c r="G158" t="n">
-        <v>576</v>
+        <v>0</v>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -6123,11 +6123,11 @@
         <v>1</v>
       </c>
       <c r="G159" t="n">
-        <v>89</v>
+        <v>0</v>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -6225,11 +6225,11 @@
         <v>1</v>
       </c>
       <c r="G162" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -6293,11 +6293,11 @@
         <v>1</v>
       </c>
       <c r="G164" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -6327,11 +6327,11 @@
         <v>1</v>
       </c>
       <c r="G165" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -6395,11 +6395,11 @@
         <v>1</v>
       </c>
       <c r="G167" t="n">
-        <v>516</v>
+        <v>0</v>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -6429,11 +6429,11 @@
         <v>1</v>
       </c>
       <c r="G168" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -6701,11 +6701,11 @@
         <v>1</v>
       </c>
       <c r="G176" t="n">
-        <v>0</v>
+        <v>950</v>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -6735,11 +6735,11 @@
         <v>1</v>
       </c>
       <c r="G177" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -6803,11 +6803,11 @@
         <v>1</v>
       </c>
       <c r="G179" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -6837,11 +6837,11 @@
         <v>1</v>
       </c>
       <c r="G180" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -6905,11 +6905,11 @@
         <v>1</v>
       </c>
       <c r="G182" t="n">
-        <v>0</v>
+        <v>156</v>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -6939,11 +6939,11 @@
         <v>1</v>
       </c>
       <c r="G183" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -7755,11 +7755,11 @@
         <v>1</v>
       </c>
       <c r="G207" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -8367,7 +8367,7 @@
         <v>1</v>
       </c>
       <c r="G225" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="H225" t="inlineStr">
         <is>
@@ -9897,7 +9897,7 @@
         <v>1</v>
       </c>
       <c r="G270" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="H270" t="inlineStr">
         <is>
@@ -10203,11 +10203,11 @@
         <v>1</v>
       </c>
       <c r="G279" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10271,11 +10271,11 @@
         <v>1</v>
       </c>
       <c r="G281" t="n">
-        <v>101</v>
+        <v>0</v>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10305,11 +10305,11 @@
         <v>1</v>
       </c>
       <c r="G282" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10373,11 +10373,11 @@
         <v>1</v>
       </c>
       <c r="G284" t="n">
-        <v>670</v>
+        <v>0</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10407,11 +10407,11 @@
         <v>1</v>
       </c>
       <c r="G285" t="n">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10509,11 +10509,11 @@
         <v>1</v>
       </c>
       <c r="G288" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10577,11 +10577,11 @@
         <v>1</v>
       </c>
       <c r="G290" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10611,11 +10611,11 @@
         <v>1</v>
       </c>
       <c r="G291" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10679,11 +10679,11 @@
         <v>1</v>
       </c>
       <c r="G293" t="n">
-        <v>941</v>
+        <v>0</v>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10713,11 +10713,11 @@
         <v>1</v>
       </c>
       <c r="G294" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10747,11 +10747,11 @@
         <v>1</v>
       </c>
       <c r="G295" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10781,11 +10781,11 @@
         <v>1</v>
       </c>
       <c r="G296" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10815,7 +10815,7 @@
         <v>1</v>
       </c>
       <c r="G297" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H297" t="inlineStr">
         <is>
@@ -10883,11 +10883,11 @@
         <v>1</v>
       </c>
       <c r="G299" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -10917,11 +10917,11 @@
         <v>1</v>
       </c>
       <c r="G300" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -10951,11 +10951,11 @@
         <v>1</v>
       </c>
       <c r="G301" t="n">
-        <v>0</v>
+        <v>9347</v>
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -10985,11 +10985,11 @@
         <v>1</v>
       </c>
       <c r="G302" t="n">
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -11019,11 +11019,11 @@
         <v>1</v>
       </c>
       <c r="G303" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -11053,11 +11053,11 @@
         <v>1</v>
       </c>
       <c r="G304" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -11121,11 +11121,11 @@
         <v>1</v>
       </c>
       <c r="G306" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -11189,11 +11189,11 @@
         <v>1</v>
       </c>
       <c r="G308" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -11427,11 +11427,11 @@
         <v>1</v>
       </c>
       <c r="G315" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11495,11 +11495,11 @@
         <v>1</v>
       </c>
       <c r="G317" t="n">
-        <v>168</v>
+        <v>0</v>
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11529,11 +11529,11 @@
         <v>1</v>
       </c>
       <c r="G318" t="n">
-        <v>178</v>
+        <v>0</v>
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11563,11 +11563,11 @@
         <v>1</v>
       </c>
       <c r="G319" t="n">
-        <v>25483</v>
+        <v>0</v>
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11597,11 +11597,11 @@
         <v>1</v>
       </c>
       <c r="G320" t="n">
-        <v>550</v>
+        <v>0</v>
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11631,11 +11631,11 @@
         <v>1</v>
       </c>
       <c r="G321" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11665,11 +11665,11 @@
         <v>1</v>
       </c>
       <c r="G322" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11733,11 +11733,11 @@
         <v>1</v>
       </c>
       <c r="G324" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H324" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11801,11 +11801,11 @@
         <v>1</v>
       </c>
       <c r="G326" t="n">
-        <v>102</v>
+        <v>0</v>
       </c>
       <c r="H326" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11835,11 +11835,11 @@
         <v>1</v>
       </c>
       <c r="G327" t="n">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11903,11 +11903,11 @@
         <v>1</v>
       </c>
       <c r="G329" t="n">
-        <v>843</v>
+        <v>0</v>
       </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11937,11 +11937,11 @@
         <v>1</v>
       </c>
       <c r="G330" t="n">
-        <v>109</v>
+        <v>0</v>
       </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -12039,7 +12039,7 @@
         <v>1</v>
       </c>
       <c r="G333" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H333" t="inlineStr">
         <is>
@@ -12107,11 +12107,11 @@
         <v>1</v>
       </c>
       <c r="G335" t="n">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -12141,11 +12141,11 @@
         <v>1</v>
       </c>
       <c r="G336" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -12209,11 +12209,11 @@
         <v>1</v>
       </c>
       <c r="G338" t="n">
-        <v>0</v>
+        <v>1035</v>
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -12243,11 +12243,11 @@
         <v>1</v>
       </c>
       <c r="G339" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="H339" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -12277,11 +12277,11 @@
         <v>1</v>
       </c>
       <c r="G340" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -12515,11 +12515,11 @@
         <v>1</v>
       </c>
       <c r="G347" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -12549,11 +12549,11 @@
         <v>1</v>
       </c>
       <c r="G348" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -12583,11 +12583,11 @@
         <v>1</v>
       </c>
       <c r="G349" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H349" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -12651,11 +12651,11 @@
         <v>1</v>
       </c>
       <c r="G351" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H351" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -12685,11 +12685,11 @@
         <v>1</v>
       </c>
       <c r="G352" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H352" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -12719,11 +12719,11 @@
         <v>1</v>
       </c>
       <c r="G353" t="n">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="H353" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -12753,11 +12753,11 @@
         <v>1</v>
       </c>
       <c r="G354" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -12821,11 +12821,11 @@
         <v>1</v>
       </c>
       <c r="G356" t="n">
-        <v>1449</v>
+        <v>0</v>
       </c>
       <c r="H356" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -12855,11 +12855,11 @@
         <v>1</v>
       </c>
       <c r="G357" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -12923,11 +12923,11 @@
         <v>1</v>
       </c>
       <c r="G359" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H359" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -12957,7 +12957,7 @@
         <v>1</v>
       </c>
       <c r="G360" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="H360" t="inlineStr">
         <is>
@@ -13331,11 +13331,11 @@
         <v>1</v>
       </c>
       <c r="G371" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -13365,11 +13365,11 @@
         <v>1</v>
       </c>
       <c r="G372" t="n">
-        <v>130</v>
+        <v>0</v>
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -13433,11 +13433,11 @@
         <v>1</v>
       </c>
       <c r="G374" t="n">
-        <v>1015</v>
+        <v>0</v>
       </c>
       <c r="H374" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -13467,11 +13467,11 @@
         <v>1</v>
       </c>
       <c r="G375" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -13569,11 +13569,11 @@
         <v>1</v>
       </c>
       <c r="G378" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -13875,11 +13875,11 @@
         <v>1</v>
       </c>
       <c r="G387" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H387" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -13943,11 +13943,11 @@
         <v>1</v>
       </c>
       <c r="G389" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="H389" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -13977,11 +13977,11 @@
         <v>1</v>
       </c>
       <c r="G390" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="H390" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -14045,11 +14045,11 @@
         <v>1</v>
       </c>
       <c r="G392" t="n">
-        <v>0</v>
+        <v>592</v>
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -14079,11 +14079,11 @@
         <v>1</v>
       </c>
       <c r="G393" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="H393" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -14181,7 +14181,7 @@
         <v>1</v>
       </c>
       <c r="G396" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="H396" t="inlineStr">
         <is>
@@ -14691,11 +14691,11 @@
         <v>1</v>
       </c>
       <c r="G411" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -14725,11 +14725,11 @@
         <v>1</v>
       </c>
       <c r="G412" t="n">
-        <v>0</v>
+        <v>86</v>
       </c>
       <c r="H412" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -14793,11 +14793,11 @@
         <v>1</v>
       </c>
       <c r="G414" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H414" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -15099,11 +15099,11 @@
         <v>1</v>
       </c>
       <c r="G423" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H423" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -15133,11 +15133,11 @@
         <v>1</v>
       </c>
       <c r="G424" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H424" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -15167,11 +15167,11 @@
         <v>1</v>
       </c>
       <c r="G425" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -15201,11 +15201,11 @@
         <v>1</v>
       </c>
       <c r="G426" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="H426" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -15269,11 +15269,11 @@
         <v>1</v>
       </c>
       <c r="G428" t="n">
-        <v>424</v>
+        <v>0</v>
       </c>
       <c r="H428" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -15303,11 +15303,11 @@
         <v>1</v>
       </c>
       <c r="G429" t="n">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -15405,11 +15405,11 @@
         <v>1</v>
       </c>
       <c r="G432" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H432" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -15439,11 +15439,11 @@
         <v>1</v>
       </c>
       <c r="G433" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H433" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -15473,11 +15473,11 @@
         <v>1</v>
       </c>
       <c r="G434" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -15507,11 +15507,11 @@
         <v>1</v>
       </c>
       <c r="G435" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="H435" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -16017,11 +16017,11 @@
         <v>1</v>
       </c>
       <c r="G450" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H450" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -16051,11 +16051,11 @@
         <v>1</v>
       </c>
       <c r="G451" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H451" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -16085,11 +16085,11 @@
         <v>1</v>
       </c>
       <c r="G452" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="H452" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -16119,11 +16119,11 @@
         <v>1</v>
       </c>
       <c r="G453" t="n">
-        <v>0</v>
+        <v>179</v>
       </c>
       <c r="H453" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -16153,11 +16153,11 @@
         <v>1</v>
       </c>
       <c r="G454" t="n">
-        <v>0</v>
+        <v>25022</v>
       </c>
       <c r="H454" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -16187,11 +16187,11 @@
         <v>1</v>
       </c>
       <c r="G455" t="n">
-        <v>0</v>
+        <v>613</v>
       </c>
       <c r="H455" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -16221,11 +16221,11 @@
         <v>1</v>
       </c>
       <c r="G456" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="H456" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -16255,11 +16255,11 @@
         <v>1</v>
       </c>
       <c r="G457" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="H457" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -16323,11 +16323,11 @@
         <v>1</v>
       </c>
       <c r="G459" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -16697,11 +16697,11 @@
         <v>1</v>
       </c>
       <c r="G470" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="H470" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -16731,11 +16731,11 @@
         <v>1</v>
       </c>
       <c r="G471" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="H471" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -16799,11 +16799,11 @@
         <v>1</v>
       </c>
       <c r="G473" t="n">
-        <v>509</v>
+        <v>0</v>
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -16833,11 +16833,11 @@
         <v>1</v>
       </c>
       <c r="G474" t="n">
-        <v>109</v>
+        <v>0</v>
       </c>
       <c r="H474" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -16935,11 +16935,11 @@
         <v>1</v>
       </c>
       <c r="G477" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -17003,11 +17003,11 @@
         <v>1</v>
       </c>
       <c r="G479" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="H479" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -17037,11 +17037,11 @@
         <v>1</v>
       </c>
       <c r="G480" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -17105,11 +17105,11 @@
         <v>1</v>
       </c>
       <c r="G482" t="n">
-        <v>475</v>
+        <v>0</v>
       </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -17139,11 +17139,11 @@
         <v>1</v>
       </c>
       <c r="G483" t="n">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -17241,7 +17241,7 @@
         <v>1</v>
       </c>
       <c r="G486" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="H486" t="inlineStr">
         <is>
@@ -17411,11 +17411,11 @@
         <v>1</v>
       </c>
       <c r="G491" t="n">
-        <v>0</v>
+        <v>982</v>
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -17445,11 +17445,11 @@
         <v>1</v>
       </c>
       <c r="G492" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -17513,11 +17513,11 @@
         <v>1</v>
       </c>
       <c r="G494" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -17547,11 +17547,11 @@
         <v>1</v>
       </c>
       <c r="G495" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -17581,11 +17581,11 @@
         <v>1</v>
       </c>
       <c r="G496" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -17615,11 +17615,11 @@
         <v>1</v>
       </c>
       <c r="G497" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -17649,11 +17649,11 @@
         <v>1</v>
       </c>
       <c r="G498" t="n">
-        <v>0</v>
+        <v>213</v>
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -17683,11 +17683,11 @@
         <v>1</v>
       </c>
       <c r="G499" t="n">
-        <v>0</v>
+        <v>26312</v>
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -17717,11 +17717,11 @@
         <v>1</v>
       </c>
       <c r="G500" t="n">
-        <v>0</v>
+        <v>499</v>
       </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -17751,11 +17751,11 @@
         <v>1</v>
       </c>
       <c r="G501" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -17785,11 +17785,11 @@
         <v>1</v>
       </c>
       <c r="G502" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -17853,7 +17853,7 @@
         <v>1</v>
       </c>
       <c r="G504" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="H504" t="inlineStr">
         <is>
@@ -18057,11 +18057,11 @@
         <v>1</v>
       </c>
       <c r="G510" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -18159,11 +18159,11 @@
         <v>1</v>
       </c>
       <c r="G513" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -18193,11 +18193,11 @@
         <v>1</v>
       </c>
       <c r="G514" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -18601,11 +18601,11 @@
         <v>1</v>
       </c>
       <c r="G526" t="n">
-        <v>0</v>
+        <v>9414</v>
       </c>
       <c r="H526" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -18635,11 +18635,11 @@
         <v>1</v>
       </c>
       <c r="G527" t="n">
-        <v>0</v>
+        <v>196</v>
       </c>
       <c r="H527" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -18669,11 +18669,11 @@
         <v>1</v>
       </c>
       <c r="G528" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H528" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -18703,11 +18703,11 @@
         <v>1</v>
       </c>
       <c r="G529" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H529" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -18771,7 +18771,7 @@
         <v>1</v>
       </c>
       <c r="G531" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="H531" t="inlineStr">
         <is>
@@ -18941,11 +18941,11 @@
         <v>1</v>
       </c>
       <c r="G536" t="n">
-        <v>0</v>
+        <v>968</v>
       </c>
       <c r="H536" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -18975,11 +18975,11 @@
         <v>1</v>
       </c>
       <c r="G537" t="n">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -19043,11 +19043,11 @@
         <v>1</v>
       </c>
       <c r="G539" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H539" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -19077,11 +19077,11 @@
         <v>1</v>
       </c>
       <c r="G540" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H540" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -19111,11 +19111,11 @@
         <v>1</v>
       </c>
       <c r="G541" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H541" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -19145,11 +19145,11 @@
         <v>1</v>
       </c>
       <c r="G542" t="n">
-        <v>0</v>
+        <v>156</v>
       </c>
       <c r="H542" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -19179,11 +19179,11 @@
         <v>1</v>
       </c>
       <c r="G543" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="H543" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -19213,11 +19213,11 @@
         <v>1</v>
       </c>
       <c r="G544" t="n">
-        <v>0</v>
+        <v>28253</v>
       </c>
       <c r="H544" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -19247,11 +19247,11 @@
         <v>1</v>
       </c>
       <c r="G545" t="n">
-        <v>0</v>
+        <v>467</v>
       </c>
       <c r="H545" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -19281,11 +19281,11 @@
         <v>1</v>
       </c>
       <c r="G546" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="H546" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -19315,11 +19315,11 @@
         <v>1</v>
       </c>
       <c r="G547" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="H547" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -19383,7 +19383,7 @@
         <v>1</v>
       </c>
       <c r="G549" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H549" t="inlineStr">
         <is>
@@ -19587,11 +19587,11 @@
         <v>1</v>
       </c>
       <c r="G555" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="H555" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -19859,11 +19859,11 @@
         <v>1</v>
       </c>
       <c r="G563" t="n">
-        <v>464</v>
+        <v>0</v>
       </c>
       <c r="H563" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -19893,11 +19893,11 @@
         <v>1</v>
       </c>
       <c r="G564" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="H564" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -19995,11 +19995,11 @@
         <v>1</v>
       </c>
       <c r="G567" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H567" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -20029,11 +20029,11 @@
         <v>1</v>
       </c>
       <c r="G568" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H568" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -20063,11 +20063,11 @@
         <v>1</v>
       </c>
       <c r="G569" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="H569" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -20097,11 +20097,11 @@
         <v>1</v>
       </c>
       <c r="G570" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="H570" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -20165,11 +20165,11 @@
         <v>1</v>
       </c>
       <c r="G572" t="n">
-        <v>485</v>
+        <v>0</v>
       </c>
       <c r="H572" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -20947,11 +20947,11 @@
         <v>1</v>
       </c>
       <c r="G595" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="H595" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -20981,11 +20981,11 @@
         <v>1</v>
       </c>
       <c r="G596" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="H596" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -21015,11 +21015,11 @@
         <v>1</v>
       </c>
       <c r="G597" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="H597" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -21083,11 +21083,11 @@
         <v>1</v>
       </c>
       <c r="G599" t="n">
-        <v>0</v>
+        <v>734</v>
       </c>
       <c r="H599" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -21117,11 +21117,11 @@
         <v>1</v>
       </c>
       <c r="G600" t="n">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="H600" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -21219,11 +21219,11 @@
         <v>1</v>
       </c>
       <c r="G603" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H603" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -21253,11 +21253,11 @@
         <v>1</v>
       </c>
       <c r="G604" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H604" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -21287,11 +21287,11 @@
         <v>1</v>
       </c>
       <c r="G605" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="H605" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -21525,11 +21525,11 @@
         <v>1</v>
       </c>
       <c r="G612" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="H612" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -21559,11 +21559,11 @@
         <v>1</v>
       </c>
       <c r="G613" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H613" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -21593,11 +21593,11 @@
         <v>1</v>
       </c>
       <c r="G614" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="H614" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -21627,11 +21627,11 @@
         <v>1</v>
       </c>
       <c r="G615" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="H615" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -21831,11 +21831,11 @@
         <v>1</v>
       </c>
       <c r="G621" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H621" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -21865,11 +21865,11 @@
         <v>1</v>
       </c>
       <c r="G622" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H622" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -21899,11 +21899,11 @@
         <v>1</v>
       </c>
       <c r="G623" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="H623" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -21933,11 +21933,11 @@
         <v>1</v>
       </c>
       <c r="G624" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="H624" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -22001,11 +22001,11 @@
         <v>1</v>
       </c>
       <c r="G626" t="n">
-        <v>0</v>
+        <v>1016</v>
       </c>
       <c r="H626" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -22035,11 +22035,11 @@
         <v>1</v>
       </c>
       <c r="G627" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="H627" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -22103,11 +22103,11 @@
         <v>1</v>
       </c>
       <c r="G629" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H629" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -22137,7 +22137,7 @@
         <v>1</v>
       </c>
       <c r="G630" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H630" t="inlineStr">
         <is>
@@ -22307,11 +22307,11 @@
         <v>1</v>
       </c>
       <c r="G635" t="n">
-        <v>536</v>
+        <v>0</v>
       </c>
       <c r="H635" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -22341,11 +22341,11 @@
         <v>1</v>
       </c>
       <c r="G636" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="H636" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -22613,11 +22613,11 @@
         <v>1</v>
       </c>
       <c r="G644" t="n">
-        <v>803</v>
+        <v>0</v>
       </c>
       <c r="H644" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -22647,11 +22647,11 @@
         <v>1</v>
       </c>
       <c r="G645" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="H645" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -22749,7 +22749,7 @@
         <v>1</v>
       </c>
       <c r="G648" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="H648" t="inlineStr">
         <is>
@@ -23089,11 +23089,11 @@
         <v>1</v>
       </c>
       <c r="G658" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="H658" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -23123,11 +23123,11 @@
         <v>1</v>
       </c>
       <c r="G659" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="H659" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -23157,11 +23157,11 @@
         <v>1</v>
       </c>
       <c r="G660" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="H660" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -23191,11 +23191,11 @@
         <v>1</v>
       </c>
       <c r="G661" t="n">
-        <v>11063</v>
+        <v>0</v>
       </c>
       <c r="H661" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -23225,11 +23225,11 @@
         <v>1</v>
       </c>
       <c r="G662" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="H662" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -23259,11 +23259,11 @@
         <v>1</v>
       </c>
       <c r="G663" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="H663" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -23293,11 +23293,11 @@
         <v>1</v>
       </c>
       <c r="G664" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H664" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -23361,11 +23361,11 @@
         <v>1</v>
       </c>
       <c r="G666" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H666" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -23395,11 +23395,11 @@
         <v>1</v>
       </c>
       <c r="G667" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H667" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -23429,11 +23429,11 @@
         <v>1</v>
       </c>
       <c r="G668" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="H668" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -23463,11 +23463,11 @@
         <v>1</v>
       </c>
       <c r="G669" t="n">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="H669" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -23531,11 +23531,11 @@
         <v>1</v>
       </c>
       <c r="G671" t="n">
-        <v>1184</v>
+        <v>0</v>
       </c>
       <c r="H671" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -23565,11 +23565,11 @@
         <v>1</v>
       </c>
       <c r="G672" t="n">
-        <v>109</v>
+        <v>0</v>
       </c>
       <c r="H672" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -23633,11 +23633,11 @@
         <v>1</v>
       </c>
       <c r="G674" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H674" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -23667,7 +23667,7 @@
         <v>1</v>
       </c>
       <c r="G675" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="H675" t="inlineStr">
         <is>
@@ -23701,11 +23701,11 @@
         <v>1</v>
       </c>
       <c r="G676" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H676" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -23735,11 +23735,11 @@
         <v>1</v>
       </c>
       <c r="G677" t="n">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="H677" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -23769,11 +23769,11 @@
         <v>1</v>
       </c>
       <c r="G678" t="n">
-        <v>0</v>
+        <v>333</v>
       </c>
       <c r="H678" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -23803,11 +23803,11 @@
         <v>1</v>
       </c>
       <c r="G679" t="n">
-        <v>0</v>
+        <v>30616</v>
       </c>
       <c r="H679" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -23837,11 +23837,11 @@
         <v>1</v>
       </c>
       <c r="G680" t="n">
-        <v>0</v>
+        <v>608</v>
       </c>
       <c r="H680" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -23871,11 +23871,11 @@
         <v>1</v>
       </c>
       <c r="G681" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="H681" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -23905,11 +23905,11 @@
         <v>1</v>
       </c>
       <c r="G682" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="H682" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -23973,11 +23973,11 @@
         <v>1</v>
       </c>
       <c r="G684" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H684" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -24007,11 +24007,11 @@
         <v>1</v>
       </c>
       <c r="G685" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="H685" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -24041,11 +24041,11 @@
         <v>1</v>
       </c>
       <c r="G686" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H686" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -24075,11 +24075,11 @@
         <v>1</v>
       </c>
       <c r="G687" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="H687" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -24143,11 +24143,11 @@
         <v>1</v>
       </c>
       <c r="G689" t="n">
-        <v>0</v>
+        <v>686</v>
       </c>
       <c r="H689" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -24177,11 +24177,11 @@
         <v>1</v>
       </c>
       <c r="G690" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="H690" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -24279,11 +24279,11 @@
         <v>1</v>
       </c>
       <c r="G693" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="H693" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -24313,11 +24313,11 @@
         <v>1</v>
       </c>
       <c r="G694" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H694" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -24347,11 +24347,11 @@
         <v>1</v>
       </c>
       <c r="G695" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="H695" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -24381,11 +24381,11 @@
         <v>1</v>
       </c>
       <c r="G696" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="H696" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -24585,11 +24585,11 @@
         <v>1</v>
       </c>
       <c r="G702" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H702" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -24619,11 +24619,11 @@
         <v>1</v>
       </c>
       <c r="G703" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H703" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -24653,11 +24653,11 @@
         <v>1</v>
       </c>
       <c r="G704" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H704" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -24687,11 +24687,11 @@
         <v>1</v>
       </c>
       <c r="G705" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="H705" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -24755,11 +24755,11 @@
         <v>1</v>
       </c>
       <c r="G707" t="n">
-        <v>0</v>
+        <v>617</v>
       </c>
       <c r="H707" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -24789,11 +24789,11 @@
         <v>1</v>
       </c>
       <c r="G708" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="H708" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -24891,7 +24891,7 @@
         <v>1</v>
       </c>
       <c r="G711" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="H711" t="inlineStr">
         <is>
@@ -25809,7 +25809,7 @@
         <v>1</v>
       </c>
       <c r="G738" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="H738" t="inlineStr">
         <is>
@@ -26013,11 +26013,11 @@
         <v>1</v>
       </c>
       <c r="G744" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="H744" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -26115,11 +26115,11 @@
         <v>1</v>
       </c>
       <c r="G747" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H747" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -26149,11 +26149,11 @@
         <v>1</v>
       </c>
       <c r="G748" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="H748" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -26183,11 +26183,11 @@
         <v>1</v>
       </c>
       <c r="G749" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H749" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -26217,11 +26217,11 @@
         <v>1</v>
       </c>
       <c r="G750" t="n">
-        <v>0</v>
+        <v>179</v>
       </c>
       <c r="H750" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -26285,11 +26285,11 @@
         <v>1</v>
       </c>
       <c r="G752" t="n">
-        <v>0</v>
+        <v>496</v>
       </c>
       <c r="H752" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -26319,11 +26319,11 @@
         <v>1</v>
       </c>
       <c r="G753" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="H753" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -26421,7 +26421,7 @@
         <v>1</v>
       </c>
       <c r="G756" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="H756" t="inlineStr">
         <is>
@@ -26455,11 +26455,11 @@
         <v>1</v>
       </c>
       <c r="G757" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H757" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -26489,11 +26489,11 @@
         <v>1</v>
       </c>
       <c r="G758" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="H758" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -26523,11 +26523,11 @@
         <v>1</v>
       </c>
       <c r="G759" t="n">
-        <v>141</v>
+        <v>0</v>
       </c>
       <c r="H759" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -26591,11 +26591,11 @@
         <v>1</v>
       </c>
       <c r="G761" t="n">
-        <v>953</v>
+        <v>0</v>
       </c>
       <c r="H761" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -26625,11 +26625,11 @@
         <v>1</v>
       </c>
       <c r="G762" t="n">
-        <v>94</v>
+        <v>0</v>
       </c>
       <c r="H762" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -26693,11 +26693,11 @@
         <v>1</v>
       </c>
       <c r="G764" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H764" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -26727,11 +26727,11 @@
         <v>1</v>
       </c>
       <c r="G765" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H765" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -26761,11 +26761,11 @@
         <v>1</v>
       </c>
       <c r="G766" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H766" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -26795,11 +26795,11 @@
         <v>1</v>
       </c>
       <c r="G767" t="n">
-        <v>161</v>
+        <v>0</v>
       </c>
       <c r="H767" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -26829,11 +26829,11 @@
         <v>1</v>
       </c>
       <c r="G768" t="n">
-        <v>185</v>
+        <v>0</v>
       </c>
       <c r="H768" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -26863,11 +26863,11 @@
         <v>1</v>
       </c>
       <c r="G769" t="n">
-        <v>26935</v>
+        <v>0</v>
       </c>
       <c r="H769" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -26897,11 +26897,11 @@
         <v>1</v>
       </c>
       <c r="G770" t="n">
-        <v>254</v>
+        <v>0</v>
       </c>
       <c r="H770" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -26931,11 +26931,11 @@
         <v>1</v>
       </c>
       <c r="G771" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="H771" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -26965,11 +26965,11 @@
         <v>1</v>
       </c>
       <c r="G772" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H772" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -27033,7 +27033,7 @@
         <v>1</v>
       </c>
       <c r="G774" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H774" t="inlineStr">
         <is>
@@ -27133,11 +27133,11 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6501</v>
+        <v>7090</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06cb838b496a29358957482b0a1175e7b736ed79996e6e714f6d056fd2c67b3e</t>
+          <t>4a40b19c73859fa2889a4fdb2a052ac494b009ed4b4356c6d7a5ee425c548785</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -27163,11 +27163,11 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3870</v>
+        <v>4135</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>60f10351a37044f81fb358192a9ea21a6c50f7cf595d724f4ce1e1f991bd78e7</t>
+          <t>baac4b25565154463d52191c994e991c3e2630cb7a1f0302ce1f47ab453af0b3</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -27193,11 +27193,11 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>205981</v>
+        <v>305384</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>e08244e149d9b9c6198be5039aea44be3a318a9d73c0b8a59841350d7161ac95</t>
+          <t>f980f5a9adcb02ee26ef894e758b79d724805f432cc55d1fccceca043362818f</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -27223,11 +27223,11 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>30278</v>
+        <v>26790</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3c70456527635006f984d469b7284338274e1a68c8ac56c4479ca5fcf3a6fcf4</t>
+          <t>66c2fbf183b95ad24c2dad91b1c79845163c5d3396c2d14f5fc89ee2f0bc0a4b</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -27253,11 +27253,11 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3914</v>
+        <v>4179</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>bc584d397582296a43a849fc7d71a4c11d739067ce5708fe21745c6c6ef64e1e</t>
+          <t>22b2e15e62e8fde2fa6b768133290fda57d7fb6a8c99c072b899111cba891cdc</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -27283,11 +27283,11 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>322</v>
+        <v>553</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>16730aa60a56cfe04717d8702f5eb3ddfcf2a2c0378faf85ad7a6e86e8c5a048</t>
+          <t>ca4f99db1fa4a73691203b2e8a57cb4aaa1bdc19f1404c09924712c99b907c2f</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -27313,11 +27313,11 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>242</v>
+        <v>220</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>197a552266f54ccdbefa33ae8d0bb7039be41e81edfe2a9fd644c7cb54f1afe7</t>
+          <t>1ff174be837f8878dfcef1d46b4f3e51e2e0fb1a9f423cfd12419c2b4eaa6a14</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -27343,11 +27343,11 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1142</v>
+        <v>1057</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>80a1f592d1095607b0c96c4a807d6927187b7c564f58a63c26ca6e847d562cdd</t>
+          <t>c241d4054f292e054818c361342b110d8dd6e67649116ef1e393b27099b167b7</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -27373,11 +27373,11 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>413</v>
+        <v>465</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>835e20cbea415f20d8f21444307502ac8cd9ba472682adcf71374da8fd20f4d9</t>
+          <t>cbc769266474375423e61a7127010f502c471baf5b1f616ff072d74438b7a242</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">

</xml_diff>